<commit_message>
Added notes to options and redesigned options page
</commit_message>
<xml_diff>
--- a/src/assets/Decision template.xlsx
+++ b/src/assets/Decision template.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Decision" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Factors" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Options" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t xml:space="preserve">Decision:</t>
   </si>
@@ -84,6 +85,12 @@
   </si>
   <si>
     <t xml:space="preserve">Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
   </si>
 </sst>
 </file>
@@ -195,37 +202,45 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -481,50 +496,50 @@
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="2" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="21.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0"/>
-      <c r="B4" s="0" t="s">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" s="7" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -572,54 +587,54 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="2" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="12.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -632,4 +647,60 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="34.37"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Abstracted options into an Option class and added hidden options
</commit_message>
<xml_diff>
--- a/src/assets/Decision template.xlsx
+++ b/src/assets/Decision template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Decision" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t xml:space="preserve">Decision:</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hidden</t>
   </si>
 </sst>
 </file>
@@ -202,7 +205,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -239,8 +242,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -654,19 +661,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="19.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="34.37"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>22</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>